<commit_message>
Dashboard: who-are-you picker, first-use guide + FAQ, read-only vault notes folder, one primary format per document (others folded), budget B2 title fix; llms.txt vault notes + folder layout
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/budget_v2.1.xlsx
+++ b/docs/budget_v2.1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CLOUD\AppData\Local\Temp\claude\c--Obsidian-60--Research\132e5da3-f94b-4205-945f-2b1468723bbb\scratchpad\a2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\nrf-status-site\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EEE3C22-820A-4977-BE7E-48560D1F5C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F756681F-0E76-4DF3-A5E4-57EB99BF4AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="9-1.소요예산 산출내역" sheetId="1" r:id="rId1"/>
@@ -159,9 +159,6 @@
     <t>소요예산 총괄표 &lt;자동입력&gt;</t>
   </si>
   <si>
-    <t>과제명: 근무규칙 전부 반영 병동 간호인력 배수표 개발: 합성 근무표 편성가능성 계산실험에 의한 산술 하한과 조합 프리미엄의 산정</t>
-  </si>
-  <si>
     <t>연구비목</t>
   </si>
   <si>
@@ -535,6 +532,10 @@
   </si>
   <si>
     <t>논문게재료 (편당 상한 추정 — 연구 1·2 원고 · 연구 3 원고, OA 포함)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>과제명: 근무 규칙을 반영한 병동 간호인력 배수표 개발: 가상근무표 시뮬레이션을 통한 추가 필요인력 산정</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1600,37 +1601,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="40" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1658,8 +1628,39 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2033,11 +2034,11 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:W88"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="3.25" style="28" customWidth="1"/>
-    <col min="2" max="2" width="5.375" style="28" customWidth="1"/>
-    <col min="3" max="3" width="28.625" style="37" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" style="28" customWidth="1"/>
+    <col min="3" max="3" width="28.58203125" style="37" customWidth="1"/>
     <col min="4" max="4" width="13.25" style="28" customWidth="1"/>
     <col min="5" max="5" width="3.75" style="28" customWidth="1"/>
     <col min="6" max="6" width="6.25" style="28" customWidth="1"/>
@@ -2047,102 +2048,102 @@
     <col min="12" max="12" width="6.25" style="28" customWidth="1"/>
     <col min="13" max="14" width="3.75" style="28" customWidth="1"/>
     <col min="15" max="15" width="13.5" style="28" customWidth="1"/>
-    <col min="16" max="16" width="10.625" style="28" customWidth="1"/>
-    <col min="17" max="17" width="31.875" style="28" customWidth="1"/>
+    <col min="16" max="16" width="10.58203125" style="28" customWidth="1"/>
+    <col min="17" max="17" width="31.83203125" style="28" customWidth="1"/>
     <col min="18" max="18" width="6.25" style="28" customWidth="1"/>
-    <col min="19" max="19" width="7.625" style="28" customWidth="1"/>
+    <col min="19" max="19" width="7.58203125" style="28" customWidth="1"/>
     <col min="20" max="20" width="9" style="28" customWidth="1"/>
     <col min="21" max="21" width="16" style="28" customWidth="1"/>
-    <col min="22" max="22" width="19.125" style="28" customWidth="1"/>
+    <col min="22" max="22" width="19.08203125" style="28" customWidth="1"/>
     <col min="23" max="23" width="18.25" style="28" customWidth="1"/>
     <col min="24" max="24" width="9" style="28" customWidth="1"/>
     <col min="25" max="16384" width="9" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="25.5" customHeight="1">
-      <c r="B1" s="169" t="s">
+      <c r="B1" s="181" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="165"/>
-      <c r="D1" s="166"/>
-      <c r="E1" s="166"/>
-      <c r="F1" s="166"/>
-      <c r="G1" s="166"/>
-      <c r="H1" s="166"/>
-      <c r="I1" s="166"/>
-      <c r="J1" s="166"/>
-      <c r="K1" s="166"/>
-      <c r="L1" s="166"/>
-      <c r="M1" s="166"/>
-      <c r="N1" s="166"/>
-      <c r="O1" s="166"/>
-      <c r="P1" s="166"/>
-      <c r="Q1" s="166"/>
-      <c r="R1" s="171" t="s">
+      <c r="C1" s="174"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
+      <c r="G1" s="175"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="175"/>
+      <c r="J1" s="175"/>
+      <c r="K1" s="175"/>
+      <c r="L1" s="175"/>
+      <c r="M1" s="175"/>
+      <c r="N1" s="175"/>
+      <c r="O1" s="175"/>
+      <c r="P1" s="175"/>
+      <c r="Q1" s="175"/>
+      <c r="R1" s="183" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="166"/>
-      <c r="T1" s="172" t="s">
+      <c r="S1" s="175"/>
+      <c r="T1" s="184" t="s">
         <v>39</v>
       </c>
-      <c r="U1" s="166"/>
-      <c r="V1" s="166"/>
-      <c r="W1" s="166"/>
+      <c r="U1" s="175"/>
+      <c r="V1" s="175"/>
+      <c r="W1" s="175"/>
     </row>
     <row r="2" spans="1:23" ht="16.5" customHeight="1">
-      <c r="B2" s="164" t="s">
+      <c r="B2" s="173" t="s">
+        <v>165</v>
+      </c>
+      <c r="C2" s="174"/>
+      <c r="D2" s="175"/>
+      <c r="E2" s="175"/>
+      <c r="F2" s="175"/>
+      <c r="G2" s="175"/>
+      <c r="H2" s="175"/>
+      <c r="I2" s="175"/>
+      <c r="J2" s="175"/>
+      <c r="K2" s="175"/>
+      <c r="L2" s="175"/>
+      <c r="M2" s="175"/>
+      <c r="N2" s="175"/>
+      <c r="O2" s="175"/>
+      <c r="P2" s="175"/>
+      <c r="Q2" s="175"/>
+      <c r="T2" s="178" t="s">
         <v>40</v>
-      </c>
-      <c r="C2" s="165"/>
-      <c r="D2" s="166"/>
-      <c r="E2" s="166"/>
-      <c r="F2" s="166"/>
-      <c r="G2" s="166"/>
-      <c r="H2" s="166"/>
-      <c r="I2" s="166"/>
-      <c r="J2" s="166"/>
-      <c r="K2" s="166"/>
-      <c r="L2" s="166"/>
-      <c r="M2" s="166"/>
-      <c r="N2" s="166"/>
-      <c r="O2" s="166"/>
-      <c r="P2" s="166"/>
-      <c r="Q2" s="166"/>
-      <c r="T2" s="162" t="s">
-        <v>41</v>
       </c>
       <c r="U2" s="158"/>
       <c r="V2" s="142" t="s">
+        <v>41</v>
+      </c>
+      <c r="W2" s="142" t="s">
         <v>42</v>
       </c>
-      <c r="W2" s="142" t="s">
+    </row>
+    <row r="3" spans="1:23">
+      <c r="B3" s="173" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="3" spans="1:23">
-      <c r="B3" s="164" t="s">
+      <c r="C3" s="174"/>
+      <c r="D3" s="175"/>
+      <c r="E3" s="175"/>
+      <c r="F3" s="175"/>
+      <c r="G3" s="175"/>
+      <c r="H3" s="175"/>
+      <c r="I3" s="175"/>
+      <c r="J3" s="175"/>
+      <c r="K3" s="175"/>
+      <c r="L3" s="175"/>
+      <c r="M3" s="175"/>
+      <c r="N3" s="175"/>
+      <c r="O3" s="175"/>
+      <c r="P3" s="175"/>
+      <c r="Q3" s="175"/>
+      <c r="T3" s="168" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="165"/>
-      <c r="D3" s="166"/>
-      <c r="E3" s="166"/>
-      <c r="F3" s="166"/>
-      <c r="G3" s="166"/>
-      <c r="H3" s="166"/>
-      <c r="I3" s="166"/>
-      <c r="J3" s="166"/>
-      <c r="K3" s="166"/>
-      <c r="L3" s="166"/>
-      <c r="M3" s="166"/>
-      <c r="N3" s="166"/>
-      <c r="O3" s="166"/>
-      <c r="P3" s="166"/>
-      <c r="Q3" s="166"/>
-      <c r="T3" s="179" t="s">
+      <c r="U3" s="138" t="s">
         <v>45</v>
-      </c>
-      <c r="U3" s="138" t="s">
-        <v>46</v>
       </c>
       <c r="V3" s="140">
         <f>O10</f>
@@ -2154,8 +2155,8 @@
       </c>
     </row>
     <row r="4" spans="1:23">
-      <c r="B4" s="170"/>
-      <c r="C4" s="165"/>
+      <c r="B4" s="182"/>
+      <c r="C4" s="174"/>
       <c r="F4" s="30"/>
       <c r="G4" s="30"/>
       <c r="H4" s="30"/>
@@ -2170,7 +2171,7 @@
       <c r="Q4" s="30"/>
       <c r="T4" s="161"/>
       <c r="U4" s="138" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="V4" s="140">
         <f>O17</f>
@@ -2183,24 +2184,24 @@
     </row>
     <row r="5" spans="1:23">
       <c r="B5" s="32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C5" s="33"/>
       <c r="K5" s="34"/>
-      <c r="L5" s="175" t="s">
-        <v>49</v>
-      </c>
-      <c r="M5" s="176"/>
-      <c r="N5" s="176"/>
+      <c r="L5" s="164" t="s">
+        <v>48</v>
+      </c>
+      <c r="M5" s="165"/>
+      <c r="N5" s="165"/>
       <c r="O5" s="35">
         <v>1500</v>
       </c>
       <c r="P5" s="30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="T5" s="161"/>
       <c r="U5" s="138" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="V5" s="140">
         <f>O26</f>
@@ -2212,31 +2213,31 @@
       </c>
     </row>
     <row r="6" spans="1:23" ht="25.5" customHeight="1" thickBot="1">
-      <c r="B6" s="177" t="s">
+      <c r="B6" s="166" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="163"/>
+      <c r="D6" s="163"/>
+      <c r="E6" s="163"/>
+      <c r="F6" s="163"/>
+      <c r="G6" s="163"/>
+      <c r="H6" s="163"/>
+      <c r="I6" s="163"/>
+      <c r="J6" s="163"/>
+      <c r="K6" s="163"/>
+      <c r="L6" s="163"/>
+      <c r="M6" s="163"/>
+      <c r="N6" s="163"/>
+      <c r="O6" s="145" t="s">
         <v>52</v>
-      </c>
-      <c r="C6" s="174"/>
-      <c r="D6" s="174"/>
-      <c r="E6" s="174"/>
-      <c r="F6" s="174"/>
-      <c r="G6" s="174"/>
-      <c r="H6" s="174"/>
-      <c r="I6" s="174"/>
-      <c r="J6" s="174"/>
-      <c r="K6" s="174"/>
-      <c r="L6" s="174"/>
-      <c r="M6" s="174"/>
-      <c r="N6" s="174"/>
-      <c r="O6" s="145" t="s">
-        <v>53</v>
       </c>
       <c r="P6" s="146"/>
       <c r="Q6" s="145" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="T6" s="161"/>
       <c r="U6" s="138" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="V6" s="140">
         <f>O31</f>
@@ -2249,7 +2250,7 @@
     </row>
     <row r="7" spans="1:23" ht="21.75" customHeight="1">
       <c r="B7" s="36" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O7" s="38">
         <f>O10+O17+O26+O31+O76</f>
@@ -2257,7 +2258,7 @@
       </c>
       <c r="T7" s="155"/>
       <c r="U7" s="138" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="V7" s="140">
         <f>O76</f>
@@ -2269,8 +2270,8 @@
       </c>
     </row>
     <row r="8" spans="1:23" ht="18" customHeight="1">
-      <c r="T8" s="163" t="s">
-        <v>58</v>
+      <c r="T8" s="179" t="s">
+        <v>57</v>
       </c>
       <c r="U8" s="158"/>
       <c r="V8" s="140">
@@ -2283,30 +2284,30 @@
       </c>
     </row>
     <row r="9" spans="1:23" ht="18" customHeight="1">
-      <c r="B9" s="182" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" s="181"/>
-      <c r="D9" s="181"/>
-      <c r="E9" s="181"/>
-      <c r="F9" s="181"/>
-      <c r="G9" s="181"/>
-      <c r="H9" s="181"/>
-      <c r="I9" s="181"/>
-      <c r="J9" s="181"/>
+      <c r="B9" s="171" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="170"/>
+      <c r="D9" s="170"/>
+      <c r="E9" s="170"/>
+      <c r="F9" s="170"/>
+      <c r="G9" s="170"/>
+      <c r="H9" s="170"/>
+      <c r="I9" s="170"/>
+      <c r="J9" s="170"/>
       <c r="K9" s="39"/>
       <c r="L9" s="39"/>
       <c r="M9" s="39"/>
       <c r="N9" s="39"/>
       <c r="O9" s="40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P9" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q9" s="42"/>
+      <c r="T9" s="168" t="s">
         <v>60</v>
-      </c>
-      <c r="Q9" s="42"/>
-      <c r="T9" s="179" t="s">
-        <v>61</v>
       </c>
       <c r="U9" s="158"/>
       <c r="V9" s="141">
@@ -2321,7 +2322,7 @@
     <row r="10" spans="1:23" ht="18" customHeight="1">
       <c r="A10" s="43"/>
       <c r="B10" s="36" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="44"/>
@@ -2344,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="Q10" s="46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="R10" s="43"/>
       <c r="S10" s="43"/>
@@ -2355,21 +2356,21 @@
     </row>
     <row r="11" spans="1:23" s="43" customFormat="1" ht="18" customHeight="1">
       <c r="C11" s="47" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="48" t="s">
+      <c r="F11" s="29" t="s">
         <v>65</v>
-      </c>
-      <c r="F11" s="29" t="s">
-        <v>66</v>
       </c>
       <c r="H11" s="29"/>
       <c r="I11" s="49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K11" s="50"/>
       <c r="L11" s="43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M11" s="49"/>
       <c r="N11" s="50"/>
@@ -2387,34 +2388,34 @@
         <v>5802624</v>
       </c>
       <c r="E12" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F12" s="123">
         <v>0.1</v>
       </c>
       <c r="G12" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="H12" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="I12" s="122">
+        <v>0</v>
+      </c>
+      <c r="J12" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="H12" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="I12" s="122">
-        <v>0</v>
-      </c>
-      <c r="J12" s="28" t="s">
+      <c r="K12" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="L12" s="122">
+        <v>0</v>
+      </c>
+      <c r="M12" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="K12" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="L12" s="122">
-        <v>0</v>
-      </c>
-      <c r="M12" s="28" t="s">
+      <c r="N12" s="54" t="s">
         <v>72</v>
-      </c>
-      <c r="N12" s="54" t="s">
-        <v>73</v>
       </c>
       <c r="O12" s="55">
         <f>D12*F12*I12*L12</f>
@@ -2439,34 +2440,34 @@
         <v>3878858</v>
       </c>
       <c r="E13" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F13" s="123">
         <v>0.05</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="H13" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="I13" s="122">
+        <v>0</v>
+      </c>
+      <c r="J13" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="H13" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="I13" s="122">
-        <v>0</v>
-      </c>
-      <c r="J13" s="28" t="s">
+      <c r="K13" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="L13" s="122">
+        <v>0</v>
+      </c>
+      <c r="M13" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="K13" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="L13" s="122">
-        <v>0</v>
-      </c>
-      <c r="M13" s="28" t="s">
+      <c r="N13" s="54" t="s">
         <v>72</v>
-      </c>
-      <c r="N13" s="54" t="s">
-        <v>73</v>
       </c>
       <c r="O13" s="55">
         <f>D13*F13*I13*L13</f>
@@ -2485,34 +2486,34 @@
         <v>2909242</v>
       </c>
       <c r="E14" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F14" s="123">
         <v>0.05</v>
       </c>
       <c r="G14" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="H14" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="122">
+        <v>0</v>
+      </c>
+      <c r="J14" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="H14" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="I14" s="122">
-        <v>0</v>
-      </c>
-      <c r="J14" s="28" t="s">
+      <c r="K14" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="L14" s="122">
+        <v>0</v>
+      </c>
+      <c r="M14" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="K14" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="L14" s="122">
-        <v>0</v>
-      </c>
-      <c r="M14" s="28" t="s">
+      <c r="N14" s="54" t="s">
         <v>72</v>
-      </c>
-      <c r="N14" s="54" t="s">
-        <v>73</v>
       </c>
       <c r="O14" s="55">
         <f>D14*F14*I14*L14</f>
@@ -2539,42 +2540,42 @@
       <c r="P15" s="63"/>
     </row>
     <row r="16" spans="1:23" ht="18" customHeight="1">
-      <c r="B16" s="180" t="s">
+      <c r="B16" s="169" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="170"/>
+      <c r="D16" s="170"/>
+      <c r="E16" s="170"/>
+      <c r="F16" s="170"/>
+      <c r="G16" s="170"/>
+      <c r="H16" s="170"/>
+      <c r="I16" s="170"/>
+      <c r="J16" s="170"/>
+      <c r="K16" s="170"/>
+      <c r="L16" s="170"/>
+      <c r="M16" s="170"/>
+      <c r="N16" s="170"/>
+      <c r="O16" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="P16" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q16" s="42"/>
+    </row>
+    <row r="17" spans="1:23" ht="18" customHeight="1">
+      <c r="B17" s="180" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="181"/>
-      <c r="D16" s="181"/>
-      <c r="E16" s="181"/>
-      <c r="F16" s="181"/>
-      <c r="G16" s="181"/>
-      <c r="H16" s="181"/>
-      <c r="I16" s="181"/>
-      <c r="J16" s="181"/>
-      <c r="K16" s="181"/>
-      <c r="L16" s="181"/>
-      <c r="M16" s="181"/>
-      <c r="N16" s="181"/>
-      <c r="O16" s="40" t="s">
-        <v>53</v>
-      </c>
-      <c r="P16" s="40" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q16" s="42"/>
-    </row>
-    <row r="17" spans="1:23" ht="18" customHeight="1">
-      <c r="B17" s="167" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" s="168"/>
-      <c r="D17" s="168"/>
-      <c r="E17" s="168"/>
-      <c r="F17" s="168"/>
-      <c r="G17" s="168"/>
-      <c r="H17" s="168"/>
-      <c r="I17" s="168"/>
-      <c r="J17" s="168"/>
-      <c r="K17" s="168"/>
+      <c r="C17" s="177"/>
+      <c r="D17" s="177"/>
+      <c r="E17" s="177"/>
+      <c r="F17" s="177"/>
+      <c r="G17" s="177"/>
+      <c r="H17" s="177"/>
+      <c r="I17" s="177"/>
+      <c r="J17" s="177"/>
+      <c r="K17" s="177"/>
       <c r="L17" s="65"/>
       <c r="M17" s="65"/>
       <c r="N17" s="65"/>
@@ -2587,16 +2588,16 @@
         <v>0</v>
       </c>
       <c r="Q17" s="46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:23" ht="18" customHeight="1">
       <c r="B18" s="66" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C18" s="67"/>
       <c r="D18" s="29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E18" s="50"/>
       <c r="F18" s="49"/>
@@ -2620,17 +2621,17 @@
     <row r="19" spans="1:23" ht="18" customHeight="1">
       <c r="B19" s="65"/>
       <c r="C19" s="121" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D19" s="122">
         <v>0</v>
       </c>
       <c r="E19" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F19" s="122"/>
       <c r="G19" s="54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H19" s="65"/>
       <c r="I19" s="65"/>
@@ -2638,7 +2639,7 @@
       <c r="L19" s="65"/>
       <c r="M19" s="65"/>
       <c r="N19" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O19" s="72">
         <f>D19*F19</f>
@@ -2649,17 +2650,17 @@
     <row r="20" spans="1:23" ht="18" customHeight="1">
       <c r="B20" s="65"/>
       <c r="C20" s="121" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D20" s="122">
         <v>0</v>
       </c>
       <c r="E20" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F20" s="122"/>
       <c r="G20" s="54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H20" s="65"/>
       <c r="I20" s="65"/>
@@ -2667,7 +2668,7 @@
       <c r="L20" s="65"/>
       <c r="M20" s="65"/>
       <c r="N20" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O20" s="72">
         <f>D20*F20</f>
@@ -2678,17 +2679,17 @@
     <row r="21" spans="1:23" ht="18" customHeight="1">
       <c r="B21" s="65"/>
       <c r="C21" s="121" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D21" s="122">
         <v>0</v>
       </c>
       <c r="E21" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F21" s="122"/>
       <c r="G21" s="54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H21" s="65"/>
       <c r="I21" s="65"/>
@@ -2696,7 +2697,7 @@
       <c r="L21" s="65"/>
       <c r="M21" s="65"/>
       <c r="N21" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O21" s="72">
         <f>D21*F21</f>
@@ -2706,7 +2707,7 @@
     </row>
     <row r="22" spans="1:23" ht="18" customHeight="1">
       <c r="B22" s="73" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C22" s="67"/>
       <c r="D22" s="68"/>
@@ -2729,21 +2730,21 @@
         <v>0</v>
       </c>
       <c r="Q22" s="29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:23" ht="18" customHeight="1">
       <c r="B23" s="65"/>
       <c r="C23" s="121" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D23" s="120"/>
       <c r="E23" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F23" s="122"/>
       <c r="G23" s="54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H23" s="65"/>
       <c r="I23" s="65"/>
@@ -2751,7 +2752,7 @@
       <c r="L23" s="65"/>
       <c r="M23" s="65"/>
       <c r="N23" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O23" s="72">
         <f>D23*F23</f>
@@ -2780,36 +2781,36 @@
       <c r="P24" s="45"/>
     </row>
     <row r="25" spans="1:23" ht="18" customHeight="1">
-      <c r="B25" s="180" t="s">
-        <v>86</v>
-      </c>
-      <c r="C25" s="181"/>
-      <c r="D25" s="181"/>
-      <c r="E25" s="181"/>
-      <c r="F25" s="181"/>
-      <c r="G25" s="181"/>
-      <c r="H25" s="181"/>
-      <c r="I25" s="181"/>
-      <c r="J25" s="181"/>
-      <c r="K25" s="181"/>
-      <c r="L25" s="181"/>
-      <c r="M25" s="181"/>
-      <c r="N25" s="181"/>
+      <c r="B25" s="169" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="170"/>
+      <c r="D25" s="170"/>
+      <c r="E25" s="170"/>
+      <c r="F25" s="170"/>
+      <c r="G25" s="170"/>
+      <c r="H25" s="170"/>
+      <c r="I25" s="170"/>
+      <c r="J25" s="170"/>
+      <c r="K25" s="170"/>
+      <c r="L25" s="170"/>
+      <c r="M25" s="170"/>
+      <c r="N25" s="170"/>
       <c r="O25" s="40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P25" s="40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="Q25" s="42"/>
     </row>
     <row r="26" spans="1:23" ht="18" customHeight="1">
       <c r="B26" s="36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C26" s="67"/>
       <c r="D26" s="29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E26" s="67"/>
       <c r="F26" s="49"/>
@@ -2830,39 +2831,39 @@
         <v>0</v>
       </c>
       <c r="Q26" s="46" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:23" ht="18" customHeight="1">
       <c r="B27" s="65"/>
       <c r="C27" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" s="122">
+        <v>0</v>
+      </c>
+      <c r="E27" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="F27" s="122">
+        <v>0</v>
+      </c>
+      <c r="G27" s="54" t="s">
+        <v>79</v>
+      </c>
+      <c r="H27" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="I27" s="122">
+        <v>0</v>
+      </c>
+      <c r="J27" s="47" t="s">
         <v>89</v>
-      </c>
-      <c r="D27" s="122">
-        <v>0</v>
-      </c>
-      <c r="E27" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="F27" s="122">
-        <v>0</v>
-      </c>
-      <c r="G27" s="54" t="s">
-        <v>80</v>
-      </c>
-      <c r="H27" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="I27" s="122">
-        <v>0</v>
-      </c>
-      <c r="J27" s="47" t="s">
-        <v>90</v>
       </c>
       <c r="L27" s="67"/>
       <c r="M27" s="67"/>
       <c r="N27" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O27" s="72">
         <f>D27*F27*I27</f>
@@ -2870,7 +2871,7 @@
       </c>
       <c r="P27" s="45"/>
       <c r="Q27" s="75" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:23" ht="18" customHeight="1">
@@ -2880,27 +2881,27 @@
         <v>0</v>
       </c>
       <c r="E28" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F28" s="122">
         <v>0</v>
       </c>
       <c r="G28" s="54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H28" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I28" s="122">
         <v>0</v>
       </c>
       <c r="J28" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L28" s="67"/>
       <c r="M28" s="67"/>
       <c r="N28" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O28" s="72">
         <f>D28*F28*I28</f>
@@ -2927,32 +2928,32 @@
     </row>
     <row r="30" spans="1:23" ht="18" customHeight="1">
       <c r="A30" s="77"/>
-      <c r="B30" s="183" t="s">
-        <v>92</v>
-      </c>
-      <c r="C30" s="181"/>
-      <c r="D30" s="181"/>
-      <c r="E30" s="181"/>
-      <c r="F30" s="181"/>
-      <c r="G30" s="181"/>
-      <c r="H30" s="181"/>
-      <c r="I30" s="181"/>
-      <c r="J30" s="181"/>
+      <c r="B30" s="172" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" s="170"/>
+      <c r="D30" s="170"/>
+      <c r="E30" s="170"/>
+      <c r="F30" s="170"/>
+      <c r="G30" s="170"/>
+      <c r="H30" s="170"/>
+      <c r="I30" s="170"/>
+      <c r="J30" s="170"/>
       <c r="K30" s="39"/>
       <c r="L30" s="39"/>
       <c r="M30" s="39"/>
       <c r="N30" s="39"/>
       <c r="O30" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="P30" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q30" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="P30" s="40" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q30" s="40" t="s">
-        <v>54</v>
-      </c>
       <c r="R30" s="40" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S30" s="77"/>
       <c r="T30" s="77"/>
@@ -2962,7 +2963,7 @@
     </row>
     <row r="31" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B31" s="36" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C31" s="67"/>
       <c r="D31" s="67"/>
@@ -2985,16 +2986,16 @@
         <v>1</v>
       </c>
       <c r="Q31" s="46" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B32" s="66" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C32" s="67"/>
       <c r="D32" s="78" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E32" s="47"/>
       <c r="F32" s="47"/>
@@ -3015,41 +3016,41 @@
         <v>0.12720000356160011</v>
       </c>
       <c r="Q32" s="46" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="A33" s="32"/>
       <c r="B33" s="86"/>
       <c r="C33" s="59" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D33" s="122">
         <v>50000</v>
       </c>
       <c r="E33" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F33" s="122">
         <v>2</v>
       </c>
       <c r="G33" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H33" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I33" s="122">
         <v>4</v>
       </c>
       <c r="J33" s="54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K33" s="54"/>
       <c r="L33" s="67"/>
       <c r="M33" s="67"/>
       <c r="N33" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O33" s="81">
         <f>D33*F33*I33</f>
@@ -3057,40 +3058,40 @@
       </c>
       <c r="P33" s="50"/>
       <c r="Q33" s="85" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B34" s="79"/>
       <c r="C34" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="D34" s="122">
+        <v>0</v>
+      </c>
+      <c r="E34" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="F34" s="122">
+        <v>0</v>
+      </c>
+      <c r="G34" s="54" t="s">
+        <v>70</v>
+      </c>
+      <c r="H34" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="I34" s="122">
+        <v>0</v>
+      </c>
+      <c r="J34" s="54" t="s">
         <v>100</v>
-      </c>
-      <c r="D34" s="122">
-        <v>0</v>
-      </c>
-      <c r="E34" s="54" t="s">
-        <v>69</v>
-      </c>
-      <c r="F34" s="122">
-        <v>0</v>
-      </c>
-      <c r="G34" s="54" t="s">
-        <v>71</v>
-      </c>
-      <c r="H34" s="54" t="s">
-        <v>69</v>
-      </c>
-      <c r="I34" s="122">
-        <v>0</v>
-      </c>
-      <c r="J34" s="54" t="s">
-        <v>101</v>
       </c>
       <c r="K34" s="54"/>
       <c r="L34" s="67"/>
       <c r="M34" s="67"/>
       <c r="N34" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O34" s="81">
         <f>D34*F34*I34</f>
@@ -3098,45 +3099,45 @@
       </c>
       <c r="P34" s="50"/>
       <c r="Q34" s="85" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="R34" s="136" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T34" s="83"/>
     </row>
     <row r="35" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B35" s="79"/>
       <c r="C35" s="59" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D35" s="137">
         <f>VLOOKUP(R35,마스터!$C$10:$E$15,3,FALSE)</f>
         <v>100000</v>
       </c>
       <c r="E35" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F35" s="122">
         <v>2</v>
       </c>
       <c r="G35" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H35" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I35" s="122">
         <v>2</v>
       </c>
       <c r="J35" s="54" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K35" s="54"/>
       <c r="L35" s="67"/>
       <c r="M35" s="67"/>
       <c r="N35" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O35" s="81">
         <f>D35*F35*I35</f>
@@ -3152,34 +3153,34 @@
     <row r="36" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B36" s="79"/>
       <c r="C36" s="59" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D36" s="80">
         <v>25000</v>
       </c>
       <c r="E36" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F36" s="122">
         <v>2</v>
       </c>
       <c r="G36" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H36" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I36" s="122">
         <v>4</v>
       </c>
       <c r="J36" s="54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K36" s="54"/>
       <c r="L36" s="67"/>
       <c r="M36" s="67"/>
       <c r="N36" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O36" s="81">
         <f>D36*F36*I36</f>
@@ -3194,34 +3195,34 @@
     <row r="37" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B37" s="79"/>
       <c r="C37" s="59" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D37" s="53">
         <v>25000</v>
       </c>
       <c r="E37" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F37" s="122">
         <v>2</v>
       </c>
       <c r="G37" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H37" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I37" s="122">
         <v>4</v>
       </c>
       <c r="J37" s="54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K37" s="54"/>
       <c r="L37" s="67"/>
       <c r="M37" s="67"/>
       <c r="N37" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O37" s="81">
         <f>D37*F37*I37</f>
@@ -3239,7 +3240,7 @@
     </row>
     <row r="38" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B38" s="66" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C38" s="67"/>
       <c r="E38" s="67"/>
@@ -3261,7 +3262,7 @@
         <v>0</v>
       </c>
       <c r="Q38" s="82" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="T38" s="28"/>
       <c r="U38" s="28"/>
@@ -3271,33 +3272,33 @@
     <row r="39" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B39" s="79"/>
       <c r="C39" s="59" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D39" s="122">
         <v>0</v>
       </c>
       <c r="E39" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F39" s="122">
         <v>0</v>
       </c>
       <c r="G39" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H39" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I39" s="122">
         <v>0</v>
       </c>
       <c r="J39" s="54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L39" s="67"/>
       <c r="M39" s="67"/>
       <c r="N39" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O39" s="81">
         <f>D39*F39*I39</f>
@@ -3305,50 +3306,50 @@
       </c>
       <c r="P39" s="50"/>
       <c r="Q39" s="85" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="R39" s="136" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="40" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="C40" s="59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D40" s="53">
         <f>VLOOKUP($R$40,마스터!$C$19:$F$34,3,FALSE)</f>
         <v>389</v>
       </c>
       <c r="E40" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F40" s="122">
         <v>0</v>
       </c>
       <c r="G40" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H40" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I40" s="122">
         <v>0</v>
       </c>
       <c r="J40" s="54" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K40" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L40" s="53">
         <f>O5</f>
         <v>1500</v>
       </c>
       <c r="M40" s="135" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N40" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O40" s="81">
         <f t="shared" ref="O40:O45" si="1">D40*F40*I40*L40</f>
@@ -3362,42 +3363,42 @@
     </row>
     <row r="41" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="C41" s="59" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D41" s="53">
         <f>VLOOKUP($R$41,마스터!$C$19:$F$34,2,FALSE)</f>
         <v>30</v>
       </c>
       <c r="E41" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F41" s="122">
         <v>0</v>
       </c>
       <c r="G41" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H41" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I41" s="122">
         <v>0</v>
       </c>
       <c r="J41" s="54" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K41" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L41" s="53">
         <f>O5</f>
         <v>1500</v>
       </c>
       <c r="M41" s="135" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N41" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O41" s="81">
         <f t="shared" si="1"/>
@@ -3412,42 +3413,42 @@
     <row r="42" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B42" s="79"/>
       <c r="C42" s="59" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D42" s="53">
         <f>VLOOKUP($R$40,마스터!$C$19:$F$34,2,FALSE)</f>
         <v>50</v>
       </c>
       <c r="E42" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F42" s="122">
         <v>0</v>
       </c>
       <c r="G42" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H42" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I42" s="122">
         <v>0</v>
       </c>
       <c r="J42" s="54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K42" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L42" s="53">
         <f>O5</f>
         <v>1500</v>
       </c>
       <c r="M42" s="135" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N42" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O42" s="81">
         <f t="shared" si="1"/>
@@ -3455,48 +3456,48 @@
       </c>
       <c r="P42" s="50"/>
       <c r="Q42" s="82" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B43" s="79"/>
       <c r="C43" s="59" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D43" s="53">
         <f>VLOOKUP($R$41,마스터!$C$19:$F$34,2,FALSE)</f>
         <v>30</v>
       </c>
       <c r="E43" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F43" s="122">
         <v>0</v>
       </c>
       <c r="G43" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H43" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I43" s="122">
         <v>0</v>
       </c>
       <c r="J43" s="54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K43" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L43" s="53">
         <f>O5</f>
         <v>1500</v>
       </c>
       <c r="M43" s="135" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N43" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O43" s="81">
         <f t="shared" si="1"/>
@@ -3508,42 +3509,42 @@
     <row r="44" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B44" s="79"/>
       <c r="C44" s="59" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D44" s="53">
         <f>VLOOKUP($R$40,마스터!$C$19:$F$34,4,FALSE)</f>
         <v>160</v>
       </c>
       <c r="E44" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F44" s="122">
         <v>0</v>
       </c>
       <c r="G44" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H44" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I44" s="122">
         <v>0</v>
       </c>
       <c r="J44" s="54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K44" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L44" s="53">
         <f>O5</f>
         <v>1500</v>
       </c>
       <c r="M44" s="135" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N44" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O44" s="81">
         <f t="shared" si="1"/>
@@ -3555,42 +3556,42 @@
     <row r="45" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B45" s="79"/>
       <c r="C45" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D45" s="53">
         <f>VLOOKUP($R$41,마스터!$C$19:$F$34,2,FALSE)</f>
         <v>30</v>
       </c>
       <c r="E45" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F45" s="122">
         <v>0</v>
       </c>
       <c r="G45" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H45" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I45" s="122">
         <v>0</v>
       </c>
       <c r="J45" s="54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K45" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L45" s="53">
         <f>O5</f>
         <v>1500</v>
       </c>
       <c r="M45" s="135" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N45" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O45" s="81">
         <f t="shared" si="1"/>
@@ -3602,7 +3603,7 @@
     <row r="46" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="A46" s="28"/>
       <c r="B46" s="90" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C46" s="91"/>
       <c r="D46" s="68"/>
@@ -3631,33 +3632,33 @@
     <row r="47" spans="1:23" ht="18" customHeight="1">
       <c r="B47" s="76"/>
       <c r="C47" s="56" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D47" s="122">
         <v>0</v>
       </c>
       <c r="E47" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F47" s="122">
         <v>0</v>
       </c>
       <c r="G47" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H47" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I47" s="122">
         <v>0</v>
       </c>
       <c r="J47" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L47" s="67"/>
       <c r="M47" s="67"/>
       <c r="N47" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O47" s="72">
         <f>D47*F47*I47</f>
@@ -3668,33 +3669,33 @@
     <row r="48" spans="1:23" ht="18" customHeight="1">
       <c r="B48" s="76"/>
       <c r="C48" s="56" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D48" s="122">
         <v>0</v>
       </c>
       <c r="E48" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F48" s="122">
         <v>0</v>
       </c>
       <c r="G48" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H48" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I48" s="122">
         <v>0</v>
       </c>
       <c r="J48" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L48" s="67"/>
       <c r="M48" s="67"/>
       <c r="N48" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O48" s="72">
         <f>D48*F48*I48</f>
@@ -3705,7 +3706,7 @@
     <row r="49" spans="1:19" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="A49" s="28"/>
       <c r="B49" s="90" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C49" s="91"/>
       <c r="D49" s="68"/>
@@ -3734,33 +3735,33 @@
     <row r="50" spans="1:19" ht="18" customHeight="1">
       <c r="B50" s="92"/>
       <c r="C50" s="56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D50" s="122">
         <v>100</v>
       </c>
       <c r="E50" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F50" s="122">
         <v>150</v>
       </c>
       <c r="G50" s="47" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H50" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I50" s="122">
         <v>10</v>
       </c>
       <c r="J50" s="47" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L50" s="67"/>
       <c r="M50" s="67"/>
       <c r="N50" s="47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O50" s="33">
         <f>D50*F50*I50</f>
@@ -3771,33 +3772,33 @@
     <row r="51" spans="1:19" ht="18" customHeight="1">
       <c r="B51" s="56"/>
       <c r="C51" s="56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D51" s="122">
         <v>100</v>
       </c>
       <c r="E51" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F51" s="122">
         <v>500</v>
       </c>
       <c r="G51" s="47" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H51" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I51" s="122">
         <v>2</v>
       </c>
       <c r="J51" s="47" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L51" s="67"/>
       <c r="M51" s="67"/>
       <c r="N51" s="47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O51" s="33">
         <f>D51*F51*I51</f>
@@ -3808,19 +3809,19 @@
     <row r="52" spans="1:19" ht="18" customHeight="1">
       <c r="B52" s="56"/>
       <c r="C52" s="56" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D52" s="122">
         <v>0</v>
       </c>
       <c r="E52" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F52" s="122">
         <v>0</v>
       </c>
       <c r="G52" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H52" s="47"/>
       <c r="I52" s="47"/>
@@ -3828,7 +3829,7 @@
       <c r="L52" s="67"/>
       <c r="M52" s="67"/>
       <c r="N52" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O52" s="33">
         <f>D52*F52</f>
@@ -3839,19 +3840,19 @@
     <row r="53" spans="1:19" ht="18" customHeight="1">
       <c r="B53" s="56"/>
       <c r="C53" s="56" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D53" s="122">
         <v>0</v>
       </c>
       <c r="E53" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F53" s="122">
         <v>0</v>
       </c>
       <c r="G53" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H53" s="47"/>
       <c r="I53" s="47"/>
@@ -3859,7 +3860,7 @@
       <c r="L53" s="67"/>
       <c r="M53" s="67"/>
       <c r="N53" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O53" s="33">
         <f>D53*F53</f>
@@ -3869,7 +3870,7 @@
     </row>
     <row r="54" spans="1:19" ht="18" customHeight="1">
       <c r="B54" s="90" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C54" s="93"/>
       <c r="D54" s="94"/>
@@ -3895,19 +3896,19 @@
     <row r="55" spans="1:19" ht="18" customHeight="1">
       <c r="B55" s="95"/>
       <c r="C55" s="56" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D55" s="122">
         <v>2800000</v>
       </c>
       <c r="E55" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F55" s="122">
         <v>2</v>
       </c>
       <c r="G55" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H55" s="47"/>
       <c r="I55" s="47"/>
@@ -3915,7 +3916,7 @@
       <c r="L55" s="67"/>
       <c r="M55" s="67"/>
       <c r="N55" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O55" s="72">
         <f>D55*F55</f>
@@ -3926,19 +3927,19 @@
     <row r="56" spans="1:19" ht="18" customHeight="1">
       <c r="B56" s="95"/>
       <c r="C56" s="56" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D56" s="122">
         <v>250000</v>
       </c>
       <c r="E56" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F56" s="122">
         <v>2</v>
       </c>
       <c r="G56" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H56" s="47"/>
       <c r="I56" s="47"/>
@@ -3946,7 +3947,7 @@
       <c r="L56" s="67"/>
       <c r="M56" s="67"/>
       <c r="N56" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O56" s="72">
         <f>D56*F56</f>
@@ -3956,7 +3957,7 @@
     </row>
     <row r="57" spans="1:19" ht="18" customHeight="1">
       <c r="B57" s="90" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C57" s="76"/>
       <c r="D57" s="97"/>
@@ -3982,33 +3983,33 @@
     <row r="58" spans="1:19" ht="18" customHeight="1">
       <c r="B58" s="95"/>
       <c r="C58" s="56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D58" s="122">
         <v>200000</v>
       </c>
       <c r="E58" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F58" s="122">
         <v>1</v>
       </c>
       <c r="G58" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H58" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I58" s="122">
         <v>2</v>
       </c>
       <c r="J58" s="54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L58" s="67"/>
       <c r="M58" s="67"/>
       <c r="N58" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O58" s="99">
         <f>D58*F58*I58</f>
@@ -4016,39 +4017,39 @@
       </c>
       <c r="P58" s="54"/>
       <c r="Q58" s="100" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="59" spans="1:19" ht="18" customHeight="1">
       <c r="B59" s="95"/>
       <c r="C59" s="56" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D59" s="122">
         <v>200000</v>
       </c>
       <c r="E59" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F59" s="124">
         <v>2</v>
       </c>
       <c r="G59" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H59" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I59" s="122">
         <v>2</v>
       </c>
       <c r="J59" s="54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L59" s="67"/>
       <c r="M59" s="67"/>
       <c r="N59" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O59" s="99">
         <f>D59*F59*I59</f>
@@ -4059,33 +4060,33 @@
     <row r="60" spans="1:19" ht="18" customHeight="1">
       <c r="B60" s="95"/>
       <c r="C60" s="56" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D60" s="122">
         <v>50000</v>
       </c>
       <c r="E60" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F60" s="122">
         <v>10</v>
       </c>
       <c r="G60" s="54" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H60" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I60" s="122">
         <v>1</v>
       </c>
       <c r="J60" s="54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L60" s="67"/>
       <c r="M60" s="67"/>
       <c r="N60" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O60" s="99">
         <f>D60*F60*I60</f>
@@ -4096,33 +4097,33 @@
     <row r="61" spans="1:19" ht="18" customHeight="1">
       <c r="B61" s="95"/>
       <c r="C61" s="56" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D61" s="122">
         <v>0</v>
       </c>
       <c r="E61" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F61" s="122">
         <v>0</v>
       </c>
       <c r="G61" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H61" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I61" s="122">
         <v>0</v>
       </c>
       <c r="J61" s="54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L61" s="67"/>
       <c r="M61" s="67"/>
       <c r="N61" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O61" s="99">
         <f>D61*F61*I61</f>
@@ -4133,33 +4134,33 @@
     <row r="62" spans="1:19" ht="18" customHeight="1">
       <c r="B62" s="95"/>
       <c r="C62" s="56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D62" s="122">
         <v>0</v>
       </c>
       <c r="E62" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F62" s="122">
         <v>0</v>
       </c>
       <c r="G62" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H62" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I62" s="122">
         <v>0</v>
       </c>
       <c r="J62" s="54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L62" s="67"/>
       <c r="M62" s="67"/>
       <c r="N62" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O62" s="99">
         <f>D62*F62*I62</f>
@@ -4167,12 +4168,12 @@
       </c>
       <c r="P62" s="54"/>
       <c r="Q62" s="100" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="63" spans="1:19" ht="18" customHeight="1">
       <c r="B63" s="90" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C63" s="91"/>
       <c r="D63" s="68"/>
@@ -4198,33 +4199,33 @@
     <row r="64" spans="1:19" ht="18" customHeight="1">
       <c r="B64" s="91"/>
       <c r="C64" s="121" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D64" s="122">
         <v>0</v>
       </c>
       <c r="E64" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F64" s="122">
         <v>0</v>
       </c>
       <c r="G64" s="47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H64" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I64" s="122">
         <v>0</v>
       </c>
       <c r="J64" s="47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L64" s="67"/>
       <c r="M64" s="67"/>
       <c r="N64" s="47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O64" s="33">
         <f>D64*F64*I64</f>
@@ -4232,39 +4233,39 @@
       </c>
       <c r="P64" s="98"/>
       <c r="Q64" s="85" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="65" spans="1:23" ht="18" customHeight="1">
       <c r="B65" s="91"/>
       <c r="C65" s="121" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D65" s="122">
         <v>0</v>
       </c>
       <c r="E65" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F65" s="122">
         <v>0</v>
       </c>
       <c r="G65" s="47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H65" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I65" s="122">
         <v>0</v>
       </c>
       <c r="J65" s="47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L65" s="67"/>
       <c r="M65" s="67"/>
       <c r="N65" s="47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O65" s="33">
         <f>D65*F65*I65</f>
@@ -4272,39 +4273,39 @@
       </c>
       <c r="P65" s="98"/>
       <c r="Q65" s="85" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="66" spans="1:23" ht="18" customHeight="1">
       <c r="B66" s="91"/>
       <c r="C66" s="63" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D66" s="122">
         <v>0</v>
       </c>
       <c r="E66" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F66" s="122">
         <v>0</v>
       </c>
       <c r="G66" s="47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H66" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I66" s="122">
         <v>0</v>
       </c>
       <c r="J66" s="47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L66" s="67"/>
       <c r="M66" s="67"/>
       <c r="N66" s="47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O66" s="33">
         <f>D66*F66*I66</f>
@@ -4312,39 +4313,39 @@
       </c>
       <c r="P66" s="98"/>
       <c r="Q66" s="85" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="67" spans="1:23" ht="18" customHeight="1">
       <c r="B67" s="91"/>
       <c r="C67" s="63" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D67" s="122">
         <v>0</v>
       </c>
       <c r="E67" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F67" s="122">
         <v>0</v>
       </c>
       <c r="G67" s="47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H67" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I67" s="122">
         <v>0</v>
       </c>
       <c r="J67" s="47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L67" s="67"/>
       <c r="M67" s="67"/>
       <c r="N67" s="47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O67" s="33">
         <f>D67*F67*I67</f>
@@ -4352,39 +4353,39 @@
       </c>
       <c r="P67" s="98"/>
       <c r="Q67" s="85" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="68" spans="1:23" ht="18" customHeight="1">
       <c r="B68" s="91"/>
       <c r="C68" s="56" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D68" s="122">
         <v>0</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F68" s="122">
         <v>0</v>
       </c>
       <c r="G68" s="47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H68" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I68" s="122">
         <v>0</v>
       </c>
       <c r="J68" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L68" s="67"/>
       <c r="M68" s="67"/>
       <c r="N68" s="47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O68" s="33">
         <f>D68*F68*I68</f>
@@ -4395,7 +4396,7 @@
     </row>
     <row r="69" spans="1:23" ht="18" customHeight="1">
       <c r="B69" s="90" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C69" s="101"/>
       <c r="D69" s="102"/>
@@ -4421,33 +4422,33 @@
     <row r="70" spans="1:23" ht="18" customHeight="1">
       <c r="B70" s="103"/>
       <c r="C70" s="53" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D70" s="122">
         <v>0</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F70" s="122">
         <v>0</v>
       </c>
       <c r="G70" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H70" s="54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I70" s="122">
         <v>2</v>
       </c>
       <c r="J70" s="54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L70" s="67"/>
       <c r="M70" s="67"/>
       <c r="N70" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O70" s="72">
         <f>D70*F70*I70</f>
@@ -4457,22 +4458,22 @@
     </row>
     <row r="71" spans="1:23" ht="18" customHeight="1">
       <c r="B71" s="95" t="s">
+        <v>147</v>
+      </c>
+      <c r="C71" s="53" t="s">
         <v>148</v>
-      </c>
-      <c r="C71" s="53" t="s">
-        <v>149</v>
       </c>
       <c r="D71" s="122">
         <v>183962</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F71" s="122">
         <v>1</v>
       </c>
       <c r="G71" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H71" s="47"/>
       <c r="I71" s="47"/>
@@ -4480,7 +4481,7 @@
       <c r="L71" s="67"/>
       <c r="M71" s="67"/>
       <c r="N71" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O71" s="72">
         <f>D71*F71</f>
@@ -4490,10 +4491,10 @@
     </row>
     <row r="72" spans="1:23" ht="18" customHeight="1">
       <c r="B72" s="144" t="s">
+        <v>149</v>
+      </c>
+      <c r="C72" s="143" t="s">
         <v>150</v>
-      </c>
-      <c r="C72" s="143" t="s">
-        <v>151</v>
       </c>
       <c r="D72" s="122"/>
       <c r="E72" s="47"/>
@@ -4511,19 +4512,19 @@
     <row r="73" spans="1:23" ht="18" customHeight="1">
       <c r="B73" s="95"/>
       <c r="C73" s="53" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D73" s="122">
         <v>0</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F73" s="122">
         <v>0</v>
       </c>
       <c r="G73" s="47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H73" s="47"/>
       <c r="I73" s="47"/>
@@ -4531,7 +4532,7 @@
       <c r="L73" s="67"/>
       <c r="M73" s="67"/>
       <c r="N73" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O73" s="72">
         <f>D73*F73</f>
@@ -4558,29 +4559,29 @@
     </row>
     <row r="75" spans="1:23" ht="18" customHeight="1">
       <c r="A75" s="77"/>
-      <c r="B75" s="180" t="s">
+      <c r="B75" s="169" t="s">
+        <v>151</v>
+      </c>
+      <c r="C75" s="170"/>
+      <c r="D75" s="170"/>
+      <c r="E75" s="170"/>
+      <c r="F75" s="170"/>
+      <c r="G75" s="170"/>
+      <c r="H75" s="170"/>
+      <c r="I75" s="170"/>
+      <c r="J75" s="170"/>
+      <c r="K75" s="170"/>
+      <c r="L75" s="170"/>
+      <c r="M75" s="170"/>
+      <c r="N75" s="170"/>
+      <c r="O75" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="P75" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q75" s="105" t="s">
         <v>152</v>
-      </c>
-      <c r="C75" s="181"/>
-      <c r="D75" s="181"/>
-      <c r="E75" s="181"/>
-      <c r="F75" s="181"/>
-      <c r="G75" s="181"/>
-      <c r="H75" s="181"/>
-      <c r="I75" s="181"/>
-      <c r="J75" s="181"/>
-      <c r="K75" s="181"/>
-      <c r="L75" s="181"/>
-      <c r="M75" s="181"/>
-      <c r="N75" s="181"/>
-      <c r="O75" s="40" t="s">
-        <v>53</v>
-      </c>
-      <c r="P75" s="40" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q75" s="105" t="s">
-        <v>153</v>
       </c>
       <c r="R75" s="77"/>
       <c r="S75" s="77"/>
@@ -4590,10 +4591,10 @@
       <c r="W75" s="77"/>
     </row>
     <row r="76" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
-      <c r="B76" s="184" t="s">
-        <v>154</v>
-      </c>
-      <c r="C76" s="168"/>
+      <c r="B76" s="176" t="s">
+        <v>153</v>
+      </c>
+      <c r="C76" s="177"/>
       <c r="D76" s="67"/>
       <c r="E76" s="67"/>
       <c r="F76" s="67"/>
@@ -4614,34 +4615,34 @@
         <v>0</v>
       </c>
       <c r="Q76" s="82" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="77" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B77" s="126"/>
       <c r="C77" s="121" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D77" s="127">
         <v>0</v>
       </c>
       <c r="E77" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F77" s="122">
         <v>1</v>
       </c>
       <c r="G77" s="122" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H77" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I77" s="122">
         <v>1</v>
       </c>
       <c r="J77" s="122" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K77" s="67"/>
       <c r="L77" s="67"/>
@@ -4653,34 +4654,34 @@
       </c>
       <c r="P77" s="71"/>
       <c r="Q77" s="75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="78" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B78" s="126"/>
       <c r="C78" s="121" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D78" s="127">
         <v>0</v>
       </c>
       <c r="E78" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F78" s="122">
         <v>1</v>
       </c>
       <c r="G78" s="122" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H78" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I78" s="122">
         <v>1</v>
       </c>
       <c r="J78" s="122" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K78" s="67"/>
       <c r="L78" s="67"/>
@@ -4692,34 +4693,34 @@
       </c>
       <c r="P78" s="71"/>
       <c r="Q78" s="75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="79" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B79" s="126"/>
       <c r="C79" s="121" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D79" s="127">
         <v>0</v>
       </c>
       <c r="E79" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F79" s="122">
         <v>1</v>
       </c>
       <c r="G79" s="122" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H79" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I79" s="122">
         <v>1</v>
       </c>
       <c r="J79" s="122" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K79" s="67"/>
       <c r="L79" s="67"/>
@@ -4731,34 +4732,34 @@
       </c>
       <c r="P79" s="71"/>
       <c r="Q79" s="75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="80" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B80" s="126"/>
       <c r="C80" s="121" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D80" s="127">
         <v>0</v>
       </c>
       <c r="E80" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F80" s="122">
         <v>1</v>
       </c>
       <c r="G80" s="122" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H80" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I80" s="122">
         <v>1</v>
       </c>
       <c r="J80" s="122" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K80" s="50"/>
       <c r="L80" s="67"/>
@@ -4770,34 +4771,34 @@
       </c>
       <c r="P80" s="71"/>
       <c r="Q80" s="75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="81" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
       <c r="B81" s="126"/>
       <c r="C81" s="121" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D81" s="127">
         <v>0</v>
       </c>
       <c r="E81" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F81" s="122">
         <v>1</v>
       </c>
       <c r="G81" s="122" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H81" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I81" s="122">
         <v>1</v>
       </c>
       <c r="J81" s="122" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K81" s="50"/>
       <c r="L81" s="67"/>
@@ -4809,7 +4810,7 @@
       </c>
       <c r="P81" s="71"/>
       <c r="Q81" s="75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="82" spans="1:23" s="77" customFormat="1" ht="18" customHeight="1">
@@ -4838,36 +4839,36 @@
       <c r="W82" s="28"/>
     </row>
     <row r="83" spans="1:23" ht="24" customHeight="1" thickBot="1">
-      <c r="B83" s="173" t="s">
-        <v>161</v>
-      </c>
-      <c r="C83" s="174"/>
-      <c r="D83" s="174"/>
-      <c r="E83" s="174"/>
-      <c r="F83" s="174"/>
-      <c r="G83" s="174"/>
-      <c r="H83" s="174"/>
-      <c r="I83" s="174"/>
-      <c r="J83" s="174"/>
-      <c r="K83" s="174"/>
-      <c r="L83" s="174"/>
-      <c r="M83" s="174"/>
-      <c r="N83" s="174"/>
+      <c r="B83" s="162" t="s">
+        <v>160</v>
+      </c>
+      <c r="C83" s="163"/>
+      <c r="D83" s="163"/>
+      <c r="E83" s="163"/>
+      <c r="F83" s="163"/>
+      <c r="G83" s="163"/>
+      <c r="H83" s="163"/>
+      <c r="I83" s="163"/>
+      <c r="J83" s="163"/>
+      <c r="K83" s="163"/>
+      <c r="L83" s="163"/>
+      <c r="M83" s="163"/>
+      <c r="N83" s="163"/>
       <c r="O83" s="147" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P83" s="147"/>
       <c r="Q83" s="145" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="84" spans="1:23" ht="18" customHeight="1">
       <c r="B84" s="36" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C84" s="65"/>
       <c r="D84" s="48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E84" s="65"/>
       <c r="F84" s="65"/>
@@ -4888,14 +4889,14 @@
     <row r="85" spans="1:23" ht="18" customHeight="1">
       <c r="B85" s="92"/>
       <c r="C85" s="56" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D85" s="109">
         <f>O7</f>
         <v>9433962</v>
       </c>
       <c r="E85" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F85" s="110">
         <v>0.06</v>
@@ -4907,7 +4908,7 @@
       <c r="L85" s="65"/>
       <c r="M85" s="65"/>
       <c r="N85" s="101" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O85" s="112">
         <f>D85*0.06</f>
@@ -4934,22 +4935,22 @@
       <c r="P86" s="114"/>
     </row>
     <row r="87" spans="1:23" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B87" s="178" t="s">
-        <v>164</v>
-      </c>
-      <c r="C87" s="174"/>
-      <c r="D87" s="174"/>
-      <c r="E87" s="174"/>
-      <c r="F87" s="174"/>
-      <c r="G87" s="174"/>
-      <c r="H87" s="174"/>
-      <c r="I87" s="174"/>
-      <c r="J87" s="174"/>
-      <c r="K87" s="174"/>
-      <c r="L87" s="174"/>
-      <c r="M87" s="174"/>
+      <c r="B87" s="167" t="s">
+        <v>163</v>
+      </c>
+      <c r="C87" s="163"/>
+      <c r="D87" s="163"/>
+      <c r="E87" s="163"/>
+      <c r="F87" s="163"/>
+      <c r="G87" s="163"/>
+      <c r="H87" s="163"/>
+      <c r="I87" s="163"/>
+      <c r="J87" s="163"/>
+      <c r="K87" s="163"/>
+      <c r="L87" s="163"/>
+      <c r="M87" s="163"/>
       <c r="N87" s="115" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O87" s="116">
         <f>O7+O84</f>
@@ -4963,6 +4964,14 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="B2:Q2"/>
+    <mergeCell ref="B17:K17"/>
+    <mergeCell ref="B1:Q1"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="T1:W1"/>
     <mergeCell ref="B83:N83"/>
     <mergeCell ref="L5:N5"/>
     <mergeCell ref="B6:N6"/>
@@ -4976,14 +4985,6 @@
     <mergeCell ref="B30:J30"/>
     <mergeCell ref="B3:Q3"/>
     <mergeCell ref="B76:C76"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="T8:U8"/>
-    <mergeCell ref="B2:Q2"/>
-    <mergeCell ref="B17:K17"/>
-    <mergeCell ref="B1:Q1"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="T1:W1"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="P22">
@@ -5015,11 +5016,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="33.25" style="148" customWidth="1"/>
-    <col min="2" max="4" width="30.125" style="148" customWidth="1"/>
-    <col min="5" max="6" width="18.125" style="148" customWidth="1"/>
+    <col min="2" max="4" width="30.08203125" style="148" customWidth="1"/>
+    <col min="5" max="6" width="18.08203125" style="148" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="22.5" customHeight="1">

</xml_diff>